<commit_message>
[feat/ASP-7924-Lesotho-Device-and-Sites-Summary-Report-improvement-needed] Change the columns to match the GxAlert report in the Lesotho Device Short Summary Report.
</commit_message>
<xml_diff>
--- a/api/templates/device_short_summary_report/en.xlsx
+++ b/api/templates/device_short_summary_report/en.xlsx
@@ -1,56 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11214"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_short_summary_report/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFDC3BC-D00B-A649-9F30-A477CFB86370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Device and Site Summary Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Device and Site Summary Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Device and Site Summary Report</t>
-  </si>
-  <si>
-    <t>Dates: &lt;Dates&gt;</t>
-  </si>
-  <si>
-    <t>&lt;StatesLabel&gt;: &lt;States&gt;</t>
-  </si>
-  <si>
-    <t>&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
-  </si>
-  <si>
-    <t>&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
-  </si>
-  <si>
-    <t>&lt;AssaysLabel&gt;: &lt;Assays&gt;</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+  <si>
+    <t xml:space="preserve">Device and Site Summary Report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dates: &lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;StatesLabel&gt;: &lt;States&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;AssaysLabel&gt;: &lt;Assays&gt;</t>
   </si>
   <si>
     <t>&lt;Table&gt;</t>
@@ -65,16 +48,61 @@
     <t>Total</t>
   </si>
   <si>
+    <t>MTB-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MTB+ Trace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MTB+ Rif-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MTB+ Rif+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MTB+ Rif?</t>
+  </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Result</t>
+  </si>
+  <si>
+    <t>Errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error Percentage</t>
+  </si>
+  <si>
     <t>&lt;name&gt;</t>
   </si>
   <si>
     <t>&lt;stateName&gt;</t>
   </si>
   <si>
-    <t>&lt;totalXpertTests&gt;</t>
-  </si>
-  <si>
-    <t>#SUM_DYNAMIC</t>
+    <t>&lt;mtbNotDetected&gt;</t>
+  </si>
+  <si>
+    <t>&lt;mtbTraceDetected&gt;</t>
+  </si>
+  <si>
+    <t>&lt;mtbDetectedRifNotDetected&gt;</t>
+  </si>
+  <si>
+    <t>&lt;mtbDetectedRifDetected&gt;</t>
+  </si>
+  <si>
+    <t>&lt;mtbDetectedRifIndeterminate&gt;</t>
+  </si>
+  <si>
+    <t>&lt;mtbInvalid&gt;</t>
+  </si>
+  <si>
+    <t>&lt;mtbNoResult&gt;</t>
+  </si>
+  <si>
+    <t>&lt;mtbError&gt;</t>
   </si>
   <si>
     <t>Totals</t>
@@ -83,57 +111,47 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
+      <sz val="12.000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color rgb="FF000000"/>
+      <sz val="16.000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
+      <sz val="12.000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="12.000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
+      <sz val="12.000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
+      <sz val="12.000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -151,87 +169,142 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="medium">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </left>
       <right style="medium">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </right>
       <top style="medium">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="none"/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </right>
-      <top/>
+      <top style="none"/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
+      </left>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin">
+        <color auto="1"/>
       </right>
       <top style="medium">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="none"/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="13">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="2" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="4" fillId="2" borderId="2" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="3" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="4" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf fontId="5" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="5" fillId="0" borderId="5" numFmtId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf fontId="6" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -239,22 +312,18 @@
   <dxfs count="1">
     <dxf>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <fgColor rgb="FF00B0F0"/>
+          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Table Style 1" pivot="0" count="1" xr9:uid="{19082F53-8A79-6F4D-9D2A-0030ECE45304}">
-      <tableStyleElement type="wholeTable" dxfId="0"/>
+    <tableStyle name="Table Style 1" pivot="0" count="1">
+      <tableStyleElement type="wholeTable" size="1" dxfId="0"/>
     </tableStyle>
   </tableStyles>
-  <colors>
-    <mruColors>
-      <color rgb="FFABEBEF"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -266,8 +335,291 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -324,7 +676,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -350,7 +702,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -427,7 +779,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -458,93 +810,177 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
+    <col customWidth="1" min="1" max="2" width="27"/>
+    <col customWidth="1" min="3" max="3" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="27.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="67.5" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>9</v>
       </c>
+      <c r="D8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>10</v>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>12</v>
+        <v>20</v>
+      </c>
+      <c r="C9" s="8" t="e">
+        <f>D9+E9+F9+G9+H9+I9+J9+K9</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="L9" s="9" t="e">
+        <f>IF(C9=0,0,K9/C9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9">
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="12" t="e">
         <f>SUM(C$9:C9)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D10" s="12">
+        <f>SUM(D$9:D9)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>13</v>
+      <c r="E10" s="12">
+        <f>SUM(E$9:E9)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="12">
+        <f>SUM(F$9:F9)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="12">
+        <f>SUM(G$9:G9)</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="12">
+        <f>SUM(H$9:H9)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="12">
+        <f>SUM(I$9:I9)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="12">
+        <f>SUM(J$9:J9)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="12">
+        <f>SUM(K$9:K9)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
-  <pageSetup orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;Cffffff&amp;A</oddHeader>
     <oddFooter>&amp;CffffffPage &amp;P</oddFooter>

</xml_diff>

<commit_message>
[feat/HD-15837-Ukraine-Customized-Report-for-GeneXpert-Ultra-Assay-in-Aspect] Fixed Device and Site short summary report template
</commit_message>
<xml_diff>
--- a/api/templates/device_short_summary_report/en.xlsx
+++ b/api/templates/device_short_summary_report/en.xlsx
@@ -1,15 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09343F4F-985B-204B-B119-F97E6813C26B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="760" windowWidth="20960" windowHeight="12640"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Device and Site Summary Report" state="visible" r:id="rId4"/>
+    <sheet name="Device and Site Summary Report" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Device and Site Summary Report'!$A$1:$M$11</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -76,7 +93,7 @@
     <t>Errors</t>
   </si>
   <si>
-    <t xml:space="preserve">Error
+    <t>Error
 Percentage</t>
   </si>
   <si>
@@ -119,62 +136,63 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm"/>
-    <numFmt numFmtId="165" formatCode="[$-409]mmmm d&quot;, &quot;yyyy"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <family val="2"/>
       <sz val="16"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <name val="Calibri"/>
-    </font>
-    <font>
       <family val="2"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <color theme="1"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -191,7 +209,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -200,45 +218,59 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium"/>
-      <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium"/>
-      <right/>
-      <top style="medium"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="medium"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="medium"/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="medium"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -253,16 +285,24 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,87 +517,87 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="11.1640625"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="19.1640625" customWidth="1"/>
     <col min="2" max="2" width="36.83203125" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="13" max="13" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" ht="67.5" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K9" s="5" t="s">
@@ -566,95 +606,103 @@
       <c r="L9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="M9" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="8" t="e">
-        <f>E9+F9+G9+H9+I9+J9+K9+L9</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E10" s="8" t="s">
+      <c r="D10" s="9">
+        <f>SUM(E10:L10)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="K10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L10" s="8" t="s">
+      <c r="L10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="9" t="e">
-        <f>IF(D9&gt;0,L9/D9,0)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="M10" s="11">
+        <f>IF(D10&gt;0,L10/D10,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11" t="e">
-        <f>SUM(D$9:D9)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E11" s="11">
-        <f>SUM(E$9:E9)</f>
-      </c>
-      <c r="F11" s="11">
-        <f>SUM(F$9:F9)</f>
-      </c>
-      <c r="G11" s="11">
-        <f>SUM(G$9:G9)</f>
-      </c>
-      <c r="H11" s="11">
-        <f>SUM(H$9:H9)</f>
-      </c>
-      <c r="I11" s="11">
-        <f>SUM(I$9:I9)</f>
-      </c>
-      <c r="J11" s="11">
-        <f>SUM(J$9:J9)</f>
-      </c>
-      <c r="K11" s="11">
-        <f>SUM(K$9:K9)</f>
-      </c>
-      <c r="L11" s="11">
-        <f>SUM(L$9:L9)</f>
-      </c>
-      <c r="M11" s="12" t="e">
-        <f>IF(D10&gt;0,L10/D10,0)</f>
-        <v>#VALUE!</v>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="10">
+        <f>SUM(D$10:D10)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="10">
+        <f>SUM(E$10:E10)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="10">
+        <f>SUM(F$10:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="10">
+        <f>SUM(G$10:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="10">
+        <f>SUM(H$10:H10)</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="10">
+        <f>SUM(I$10:I10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="10">
+        <f>SUM(J$10:J10)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="10">
+        <f>SUM(K$10:K10)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="10">
+        <f>SUM(L$10:L10)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="12">
+        <f>IF(D11&gt;0,L11/D11,0)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7875000000000001" right="0.7875000000000001" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <headerFooter>
     <oddHeader>&amp;Cffffff&amp;A</oddHeader>
     <oddFooter>&amp;CffffffPage &amp;P</oddFooter>

</xml_diff>